<commit_message>
update enemies wave excel
</commit_message>
<xml_diff>
--- a/Assets/Configs/SpawnRoots.xlsx
+++ b/Assets/Configs/SpawnRoots.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Assignment\FoodGuardian\Project3D\Assets\Configs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BA25F50-99B0-433E-AAE4-A6D9AC548581}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F76DEA35-1678-4D56-8359-6F1751128473}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -395,7 +395,7 @@
         <v>0.6</v>
       </c>
       <c r="E2">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -412,7 +412,7 @@
         <v>0.6</v>
       </c>
       <c r="E3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -429,7 +429,7 @@
         <v>1</v>
       </c>
       <c r="E4">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -446,7 +446,7 @@
         <v>1</v>
       </c>
       <c r="E5">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -463,7 +463,7 @@
         <v>1</v>
       </c>
       <c r="E6">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -480,7 +480,7 @@
         <v>2</v>
       </c>
       <c r="E7">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -497,7 +497,7 @@
         <v>2</v>
       </c>
       <c r="E8">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -514,7 +514,7 @@
         <v>2</v>
       </c>
       <c r="E9">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -531,7 +531,7 @@
         <v>3</v>
       </c>
       <c r="E10">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -548,7 +548,7 @@
         <v>3</v>
       </c>
       <c r="E11">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -565,7 +565,7 @@
         <v>0.6</v>
       </c>
       <c r="E12">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -582,7 +582,7 @@
         <v>0.6</v>
       </c>
       <c r="E13">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -596,7 +596,7 @@
         <v>1002</v>
       </c>
       <c r="D14">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="E14">
         <v>2</v>
@@ -613,7 +613,7 @@
         <v>1002</v>
       </c>
       <c r="D15">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="E15">
         <v>2</v>
@@ -630,7 +630,7 @@
         <v>1002</v>
       </c>
       <c r="D16">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="E16">
         <v>2</v>
@@ -647,10 +647,10 @@
         <v>1002</v>
       </c>
       <c r="D17">
-        <v>0.6</v>
+        <v>2</v>
       </c>
       <c r="E17">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -664,10 +664,10 @@
         <v>1002</v>
       </c>
       <c r="D18">
-        <v>0.6</v>
+        <v>2</v>
       </c>
       <c r="E18">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -681,10 +681,10 @@
         <v>1002</v>
       </c>
       <c r="D19">
-        <v>0.6</v>
+        <v>2</v>
       </c>
       <c r="E19">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -698,10 +698,10 @@
         <v>1002</v>
       </c>
       <c r="D20">
-        <v>0.6</v>
+        <v>3</v>
       </c>
       <c r="E20">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -715,10 +715,10 @@
         <v>1002</v>
       </c>
       <c r="D21">
-        <v>0.6</v>
+        <v>3</v>
       </c>
       <c r="E21">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -735,7 +735,7 @@
         <v>0.6</v>
       </c>
       <c r="E22">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -752,7 +752,7 @@
         <v>0.6</v>
       </c>
       <c r="E23">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -766,10 +766,10 @@
         <v>1003</v>
       </c>
       <c r="D24">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="E24">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -783,10 +783,10 @@
         <v>1003</v>
       </c>
       <c r="D25">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="E25">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -800,10 +800,10 @@
         <v>1003</v>
       </c>
       <c r="D26">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="E26">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -817,7 +817,7 @@
         <v>1003</v>
       </c>
       <c r="D27">
-        <v>0.6</v>
+        <v>2</v>
       </c>
       <c r="E27">
         <v>2</v>
@@ -834,7 +834,7 @@
         <v>1003</v>
       </c>
       <c r="D28">
-        <v>0.6</v>
+        <v>2</v>
       </c>
       <c r="E28">
         <v>2</v>
@@ -851,7 +851,7 @@
         <v>1003</v>
       </c>
       <c r="D29">
-        <v>0.6</v>
+        <v>2</v>
       </c>
       <c r="E29">
         <v>2</v>
@@ -868,10 +868,10 @@
         <v>1003</v>
       </c>
       <c r="D30">
-        <v>0.6</v>
+        <v>3</v>
       </c>
       <c r="E30">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="31" spans="1:5">
@@ -885,10 +885,10 @@
         <v>1003</v>
       </c>
       <c r="D31">
-        <v>0.6</v>
+        <v>3</v>
       </c>
       <c r="E31">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>